<commit_message>
All ECM logic finished
</commit_message>
<xml_diff>
--- a/DATA.xlsx
+++ b/DATA.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E141"/>
+  <dimension ref="A1:D141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,12 +446,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Среднемесячная номинальная начисленная заработная плата, руб. </t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Коэффициент естественного прироста населения (на 1000 населения), человек</t>
+          <t>Реальные денежные доходы населения, в % к СППГ</t>
         </is>
       </c>
     </row>
@@ -468,10 +463,7 @@
         <v>108.73</v>
       </c>
       <c r="D2" t="n">
-        <v>21207.5</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-1.5</v>
+        <v>100.4</v>
       </c>
     </row>
     <row r="3">
@@ -487,10 +479,7 @@
         <v>122.21</v>
       </c>
       <c r="D3" t="n">
-        <v>24202.1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>-1.2</v>
+        <v>112.9</v>
       </c>
     </row>
     <row r="4">
@@ -506,10 +495,7 @@
         <v>105.49</v>
       </c>
       <c r="D4" t="n">
-        <v>26789</v>
-      </c>
-      <c r="E4" t="n">
-        <v>-0.4</v>
+        <v>113.3</v>
       </c>
     </row>
     <row r="5">
@@ -525,10 +511,7 @@
         <v>109.58</v>
       </c>
       <c r="D5" t="n">
-        <v>30541.7</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.2</v>
+        <v>104.4</v>
       </c>
     </row>
     <row r="6">
@@ -544,10 +527,7 @@
         <v>110.06</v>
       </c>
       <c r="D6" t="n">
-        <v>32397</v>
-      </c>
-      <c r="E6" t="n">
-        <v>-0.2</v>
+        <v>101.9</v>
       </c>
     </row>
     <row r="7">
@@ -563,10 +543,7 @@
         <v>102.39</v>
       </c>
       <c r="D7" t="n">
-        <v>32902</v>
-      </c>
-      <c r="E7" t="n">
-        <v>-0.5</v>
+        <v>96.09999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -582,10 +559,7 @@
         <v>99.93000000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>33837</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-0.8</v>
+        <v>92.09999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -601,10 +575,7 @@
         <v>100.16</v>
       </c>
       <c r="D9" t="n">
-        <v>37368</v>
-      </c>
-      <c r="E9" t="n">
-        <v>-1.5</v>
+        <v>101.1</v>
       </c>
     </row>
     <row r="10">
@@ -620,10 +591,7 @@
         <v>111.97</v>
       </c>
       <c r="D10" t="n">
-        <v>37846.5</v>
-      </c>
-      <c r="E10" t="n">
-        <v>-2.3</v>
+        <v>102.4</v>
       </c>
     </row>
     <row r="11">
@@ -639,10 +607,7 @@
         <v>112.05</v>
       </c>
       <c r="D11" t="n">
-        <v>47234</v>
-      </c>
-      <c r="E11" t="n">
-        <v>-4.1</v>
+        <v>101.7</v>
       </c>
     </row>
     <row r="12">
@@ -658,10 +623,7 @@
         <v>121.13</v>
       </c>
       <c r="D12" t="n">
-        <v>52430</v>
-      </c>
-      <c r="E12" t="n">
-        <v>-6.3</v>
+        <v>100.4</v>
       </c>
     </row>
     <row r="13">
@@ -677,10 +639,7 @@
         <v>112.95</v>
       </c>
       <c r="D13" t="n">
-        <v>59098</v>
-      </c>
-      <c r="E13" t="n">
-        <v>-9.1</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14">
@@ -696,10 +655,7 @@
         <v>109.54</v>
       </c>
       <c r="D14" t="n">
-        <v>65863.89999999999</v>
-      </c>
-      <c r="E14" t="n">
-        <v>-5.7</v>
+        <v>109.7</v>
       </c>
     </row>
     <row r="15">
@@ -715,10 +671,7 @@
         <v>111.58</v>
       </c>
       <c r="D15" t="n">
-        <v>72998.8</v>
-      </c>
-      <c r="E15" t="n">
-        <v>-4.9</v>
+        <v>99.90000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -734,10 +687,7 @@
         <v>111.9</v>
       </c>
       <c r="D16" t="n">
-        <v>19718</v>
-      </c>
-      <c r="E16" t="n">
-        <v>-1.9</v>
+        <v>103.5</v>
       </c>
     </row>
     <row r="17">
@@ -753,10 +703,7 @@
         <v>117.64</v>
       </c>
       <c r="D17" t="n">
-        <v>22927.5</v>
-      </c>
-      <c r="E17" t="n">
-        <v>-1.3</v>
+        <v>96.8</v>
       </c>
     </row>
     <row r="18">
@@ -772,10 +719,7 @@
         <v>119.27</v>
       </c>
       <c r="D18" t="n">
-        <v>25067</v>
-      </c>
-      <c r="E18" t="n">
-        <v>-1.1</v>
+        <v>102.2</v>
       </c>
     </row>
     <row r="19">
@@ -791,10 +735,7 @@
         <v>105.58</v>
       </c>
       <c r="D19" t="n">
-        <v>27357.7</v>
-      </c>
-      <c r="E19" t="n">
-        <v>-0.9</v>
+        <v>101.5</v>
       </c>
     </row>
     <row r="20">
@@ -810,10 +751,7 @@
         <v>107.73</v>
       </c>
       <c r="D20" t="n">
-        <v>29439</v>
-      </c>
-      <c r="E20" t="n">
-        <v>-1</v>
+        <v>97.7</v>
       </c>
     </row>
     <row r="21">
@@ -829,10 +767,7 @@
         <v>95.53</v>
       </c>
       <c r="D21" t="n">
-        <v>30896</v>
-      </c>
-      <c r="E21" t="n">
-        <v>-1.4</v>
+        <v>93.7</v>
       </c>
     </row>
     <row r="22">
@@ -848,10 +783,7 @@
         <v>96.31999999999999</v>
       </c>
       <c r="D22" t="n">
-        <v>32165</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-1.8</v>
+        <v>89.2</v>
       </c>
     </row>
     <row r="23">
@@ -867,10 +799,7 @@
         <v>97.38</v>
       </c>
       <c r="D23" t="n">
-        <v>34409</v>
-      </c>
-      <c r="E23" t="n">
-        <v>-1.6</v>
+        <v>97.2</v>
       </c>
     </row>
     <row r="24">
@@ -886,10 +815,7 @@
         <v>103.25</v>
       </c>
       <c r="D24" t="n">
-        <v>35292.48</v>
-      </c>
-      <c r="E24" t="n">
-        <v>-2</v>
+        <v>99.59999999999999</v>
       </c>
     </row>
     <row r="25">
@@ -905,10 +831,7 @@
         <v>98.23999999999999</v>
       </c>
       <c r="D25" t="n">
-        <v>42400</v>
-      </c>
-      <c r="E25" t="n">
-        <v>-3.7</v>
+        <v>101.2</v>
       </c>
     </row>
     <row r="26">
@@ -924,10 +847,7 @@
         <v>109.6</v>
       </c>
       <c r="D26" t="n">
-        <v>46237</v>
-      </c>
-      <c r="E26" t="n">
-        <v>-5.7</v>
+        <v>99.5</v>
       </c>
     </row>
     <row r="27">
@@ -943,10 +863,7 @@
         <v>128.91</v>
       </c>
       <c r="D27" t="n">
-        <v>50074.8</v>
-      </c>
-      <c r="E27" t="n">
-        <v>-8.4</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -962,10 +879,7 @@
         <v>123.15</v>
       </c>
       <c r="D28" t="n">
-        <v>56956.8</v>
-      </c>
-      <c r="E28" t="n">
-        <v>-5.7</v>
+        <v>104.5</v>
       </c>
     </row>
     <row r="29">
@@ -981,10 +895,7 @@
         <v>120.48</v>
       </c>
       <c r="D29" t="n">
-        <v>65815.3</v>
-      </c>
-      <c r="E29" t="n">
-        <v>-5.2</v>
+        <v>106.6</v>
       </c>
     </row>
     <row r="30">
@@ -1000,10 +911,7 @@
         <v>95.69</v>
       </c>
       <c r="D30" t="n">
-        <v>18684.5</v>
-      </c>
-      <c r="E30" t="n">
-        <v>2.1</v>
+        <v>103.2</v>
       </c>
     </row>
     <row r="31">
@@ -1019,10 +927,7 @@
         <v>103.48</v>
       </c>
       <c r="D31" t="n">
-        <v>21099.6</v>
-      </c>
-      <c r="E31" t="n">
-        <v>2.3</v>
+        <v>102.1</v>
       </c>
     </row>
     <row r="32">
@@ -1038,10 +943,7 @@
         <v>115.5</v>
       </c>
       <c r="D32" t="n">
-        <v>24218.5</v>
-      </c>
-      <c r="E32" t="n">
-        <v>3.1</v>
+        <v>103.1</v>
       </c>
     </row>
     <row r="33">
@@ -1057,10 +959,7 @@
         <v>108.73</v>
       </c>
       <c r="D33" t="n">
-        <v>27279.4</v>
-      </c>
-      <c r="E33" t="n">
-        <v>3.5</v>
+        <v>104.8</v>
       </c>
     </row>
     <row r="34">
@@ -1076,10 +975,7 @@
         <v>104.27</v>
       </c>
       <c r="D34" t="n">
-        <v>29319</v>
-      </c>
-      <c r="E34" t="n">
-        <v>3.6</v>
+        <v>95.40000000000001</v>
       </c>
     </row>
     <row r="35">
@@ -1095,10 +991,7 @@
         <v>96.70999999999999</v>
       </c>
       <c r="D35" t="n">
-        <v>30931</v>
-      </c>
-      <c r="E35" t="n">
-        <v>2.6</v>
+        <v>95.2</v>
       </c>
     </row>
     <row r="36">
@@ -1114,10 +1007,7 @@
         <v>102.3</v>
       </c>
       <c r="D36" t="n">
-        <v>32654</v>
-      </c>
-      <c r="E36" t="n">
-        <v>2.3</v>
+        <v>93.3</v>
       </c>
     </row>
     <row r="37">
@@ -1133,10 +1023,7 @@
         <v>100.23</v>
       </c>
       <c r="D37" t="n">
-        <v>34848</v>
-      </c>
-      <c r="E37" t="n">
-        <v>1.7</v>
+        <v>98.90000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -1152,10 +1039,7 @@
         <v>100.58</v>
       </c>
       <c r="D38" t="n">
-        <v>35272.24</v>
-      </c>
-      <c r="E38" t="n">
-        <v>0.4</v>
+        <v>102.1</v>
       </c>
     </row>
     <row r="39">
@@ -1171,10 +1055,7 @@
         <v>104.02</v>
       </c>
       <c r="D39" t="n">
-        <v>43896</v>
-      </c>
-      <c r="E39" t="n">
-        <v>-0.6</v>
+        <v>101.9</v>
       </c>
     </row>
     <row r="40">
@@ -1190,10 +1071,7 @@
         <v>116.58</v>
       </c>
       <c r="D40" t="n">
-        <v>47172</v>
-      </c>
-      <c r="E40" t="n">
-        <v>-2</v>
+        <v>99.90000000000001</v>
       </c>
     </row>
     <row r="41">
@@ -1209,10 +1087,7 @@
         <v>103.19</v>
       </c>
       <c r="D41" t="n">
-        <v>52216</v>
-      </c>
-      <c r="E41" t="n">
-        <v>-4.5</v>
+        <v>102.1</v>
       </c>
     </row>
     <row r="42">
@@ -1228,10 +1103,7 @@
         <v>102.49</v>
       </c>
       <c r="D42" t="n">
-        <v>59412.9</v>
-      </c>
-      <c r="E42" t="n">
-        <v>-2.6</v>
+        <v>107.3</v>
       </c>
     </row>
     <row r="43">
@@ -1247,10 +1119,7 @@
         <v>101.73</v>
       </c>
       <c r="D43" t="n">
-        <v>69830.3</v>
-      </c>
-      <c r="E43" t="n">
-        <v>-3.2</v>
+        <v>102.5</v>
       </c>
     </row>
     <row r="44">
@@ -1266,10 +1135,7 @@
         <v>100.76</v>
       </c>
       <c r="D44" t="n">
-        <v>35747.6</v>
-      </c>
-      <c r="E44" t="n">
-        <v>-0.6</v>
+        <v>103.2</v>
       </c>
     </row>
     <row r="45">
@@ -1285,10 +1151,7 @@
         <v>92.78</v>
       </c>
       <c r="D45" t="n">
-        <v>39325.9</v>
-      </c>
-      <c r="E45" t="n">
-        <v>0.4</v>
+        <v>99.2</v>
       </c>
     </row>
     <row r="46">
@@ -1304,10 +1167,7 @@
         <v>110.78</v>
       </c>
       <c r="D46" t="n">
-        <v>43551.9</v>
-      </c>
-      <c r="E46" t="n">
-        <v>1.4</v>
+        <v>103.6</v>
       </c>
     </row>
     <row r="47">
@@ -1323,10 +1183,7 @@
         <v>107.65</v>
       </c>
       <c r="D47" t="n">
-        <v>48628.8</v>
-      </c>
-      <c r="E47" t="n">
-        <v>1.7</v>
+        <v>104.7</v>
       </c>
     </row>
     <row r="48">
@@ -1342,10 +1199,7 @@
         <v>103.41</v>
       </c>
       <c r="D48" t="n">
-        <v>53167</v>
-      </c>
-      <c r="E48" t="n">
-        <v>1.7</v>
+        <v>102.4</v>
       </c>
     </row>
     <row r="49">
@@ -1361,10 +1215,7 @@
         <v>97.77</v>
       </c>
       <c r="D49" t="n">
-        <v>57404</v>
-      </c>
-      <c r="E49" t="n">
-        <v>1.7</v>
+        <v>97.2</v>
       </c>
     </row>
     <row r="50">
@@ -1380,10 +1231,7 @@
         <v>94.84999999999999</v>
       </c>
       <c r="D50" t="n">
-        <v>61159</v>
-      </c>
-      <c r="E50" t="n">
-        <v>1.4</v>
+        <v>94.59999999999999</v>
       </c>
     </row>
     <row r="51">
@@ -1399,10 +1247,7 @@
         <v>100.91</v>
       </c>
       <c r="D51" t="n">
-        <v>65807</v>
-      </c>
-      <c r="E51" t="n">
-        <v>1</v>
+        <v>99.59999999999999</v>
       </c>
     </row>
     <row r="52">
@@ -1418,10 +1263,7 @@
         <v>98.02</v>
       </c>
       <c r="D52" t="n">
-        <v>61739.37</v>
-      </c>
-      <c r="E52" t="n">
-        <v>-0.5</v>
+        <v>105.1</v>
       </c>
     </row>
     <row r="53">
@@ -1437,10 +1279,7 @@
         <v>107.22</v>
       </c>
       <c r="D53" t="n">
-        <v>80448</v>
-      </c>
-      <c r="E53" t="n">
-        <v>-0.5</v>
+        <v>103.9</v>
       </c>
     </row>
     <row r="54">
@@ -1456,10 +1295,7 @@
         <v>116.48</v>
       </c>
       <c r="D54" t="n">
-        <v>85623</v>
-      </c>
-      <c r="E54" t="n">
-        <v>-2.5</v>
+        <v>102.1</v>
       </c>
     </row>
     <row r="55">
@@ -1475,10 +1311,7 @@
         <v>102.67</v>
       </c>
       <c r="D55" t="n">
-        <v>93880.3</v>
-      </c>
-      <c r="E55" t="n">
-        <v>-4.8</v>
+        <v>104.3</v>
       </c>
     </row>
     <row r="56">
@@ -1494,10 +1327,7 @@
         <v>108.03</v>
       </c>
       <c r="D56" t="n">
-        <v>103539.9</v>
-      </c>
-      <c r="E56" t="n">
-        <v>-3</v>
+        <v>106</v>
       </c>
     </row>
     <row r="57">
@@ -1513,10 +1343,7 @@
         <v>100.28</v>
       </c>
       <c r="D57" t="n">
-        <v>119562.5</v>
-      </c>
-      <c r="E57" t="n">
-        <v>-1.6</v>
+        <v>103.8</v>
       </c>
     </row>
     <row r="58">
@@ -1532,10 +1359,7 @@
         <v>100.46</v>
       </c>
       <c r="D58" t="n">
-        <v>36582</v>
-      </c>
-      <c r="E58" t="n">
-        <v>-1.5</v>
+        <v>103.8</v>
       </c>
     </row>
     <row r="59">
@@ -1551,10 +1375,7 @@
         <v>108.83</v>
       </c>
       <c r="D59" t="n">
-        <v>41933.7</v>
-      </c>
-      <c r="E59" t="n">
-        <v>-1.4</v>
+        <v>98</v>
       </c>
     </row>
     <row r="60">
@@ -1570,10 +1391,7 @@
         <v>144.22</v>
       </c>
       <c r="D60" t="n">
-        <v>49667.3</v>
-      </c>
-      <c r="E60" t="n">
-        <v>-0.1</v>
+        <v>110.5</v>
       </c>
     </row>
     <row r="61">
@@ -1589,10 +1407,7 @@
         <v>120.5</v>
       </c>
       <c r="D61" t="n">
-        <v>57121.1</v>
-      </c>
-      <c r="E61" t="n">
-        <v>0.6</v>
+        <v>104.5</v>
       </c>
     </row>
     <row r="62">
@@ -1608,10 +1423,7 @@
         <v>104.07</v>
       </c>
       <c r="D62" t="n">
-        <v>62152</v>
-      </c>
-      <c r="E62" t="n">
-        <v>0.2</v>
+        <v>99.5</v>
       </c>
     </row>
     <row r="63">
@@ -1627,10 +1439,7 @@
         <v>90.06</v>
       </c>
       <c r="D63" t="n">
-        <v>65996</v>
-      </c>
-      <c r="E63" t="n">
-        <v>0.1</v>
+        <v>97.3</v>
       </c>
     </row>
     <row r="64">
@@ -1646,10 +1455,7 @@
         <v>99.73999999999999</v>
       </c>
       <c r="D64" t="n">
-        <v>69769</v>
-      </c>
-      <c r="E64" t="n">
-        <v>-0.3</v>
+        <v>93.90000000000001</v>
       </c>
     </row>
     <row r="65">
@@ -1665,10 +1471,7 @@
         <v>87.27</v>
       </c>
       <c r="D65" t="n">
-        <v>75710</v>
-      </c>
-      <c r="E65" t="n">
-        <v>-0.6</v>
+        <v>102.3</v>
       </c>
     </row>
     <row r="66">
@@ -1684,10 +1487,7 @@
         <v>101.45</v>
       </c>
       <c r="D66" t="n">
-        <v>73310.71000000001</v>
-      </c>
-      <c r="E66" t="n">
-        <v>-1.4</v>
+        <v>104.5</v>
       </c>
     </row>
     <row r="67">
@@ -1703,10 +1503,7 @@
         <v>106.04</v>
       </c>
       <c r="D67" t="n">
-        <v>94856</v>
-      </c>
-      <c r="E67" t="n">
-        <v>-2.5</v>
+        <v>103.1</v>
       </c>
     </row>
     <row r="68">
@@ -1722,10 +1519,7 @@
         <v>110</v>
       </c>
       <c r="D68" t="n">
-        <v>102843</v>
-      </c>
-      <c r="E68" t="n">
-        <v>-3.2</v>
+        <v>104.4</v>
       </c>
     </row>
     <row r="69">
@@ -1741,10 +1535,7 @@
         <v>127.7</v>
       </c>
       <c r="D69" t="n">
-        <v>112851.9</v>
-      </c>
-      <c r="E69" t="n">
-        <v>-6.4</v>
+        <v>106.1</v>
       </c>
     </row>
     <row r="70">
@@ -1760,10 +1551,7 @@
         <v>124.56</v>
       </c>
       <c r="D70" t="n">
-        <v>121461.8</v>
-      </c>
-      <c r="E70" t="n">
-        <v>-4</v>
+        <v>109.5</v>
       </c>
     </row>
     <row r="71">
@@ -1779,10 +1567,7 @@
         <v>114.49</v>
       </c>
       <c r="D71" t="n">
-        <v>134645.8</v>
-      </c>
-      <c r="E71" t="n">
-        <v>-3.8</v>
+        <v>101.7</v>
       </c>
     </row>
     <row r="72">
@@ -1798,10 +1583,7 @@
         <v>102.37</v>
       </c>
       <c r="D72" t="n">
-        <v>21888.7</v>
-      </c>
-      <c r="E72" t="n">
-        <v>-2.5</v>
+        <v>105.5</v>
       </c>
     </row>
     <row r="73">
@@ -1817,10 +1599,7 @@
         <v>109.88</v>
       </c>
       <c r="D73" t="n">
-        <v>24423</v>
-      </c>
-      <c r="E73" t="n">
-        <v>-2.1</v>
+        <v>102.9</v>
       </c>
     </row>
     <row r="74">
@@ -1836,10 +1615,7 @@
         <v>109.96</v>
       </c>
       <c r="D74" t="n">
-        <v>27444.6</v>
-      </c>
-      <c r="E74" t="n">
-        <v>-1</v>
+        <v>105.1</v>
       </c>
     </row>
     <row r="75">
@@ -1855,10 +1631,7 @@
         <v>101.29</v>
       </c>
       <c r="D75" t="n">
-        <v>29965.7</v>
-      </c>
-      <c r="E75" t="n">
-        <v>-0.8</v>
+        <v>105.3</v>
       </c>
     </row>
     <row r="76">
@@ -1874,10 +1647,7 @@
         <v>104.74</v>
       </c>
       <c r="D76" t="n">
-        <v>32431</v>
-      </c>
-      <c r="E76" t="n">
-        <v>-0.7</v>
+        <v>107.3</v>
       </c>
     </row>
     <row r="77">
@@ -1893,10 +1663,7 @@
         <v>105.68</v>
       </c>
       <c r="D77" t="n">
-        <v>33807</v>
-      </c>
-      <c r="E77" t="n">
-        <v>-0.8</v>
+        <v>97.7</v>
       </c>
     </row>
     <row r="78">
@@ -1912,10 +1679,7 @@
         <v>96.62</v>
       </c>
       <c r="D78" t="n">
-        <v>35677</v>
-      </c>
-      <c r="E78" t="n">
-        <v>-1.4</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="79">
@@ -1931,10 +1695,7 @@
         <v>99</v>
       </c>
       <c r="D79" t="n">
-        <v>38045</v>
-      </c>
-      <c r="E79" t="n">
-        <v>-2.4</v>
+        <v>99.8</v>
       </c>
     </row>
     <row r="80">
@@ -1950,10 +1711,7 @@
         <v>106.96</v>
       </c>
       <c r="D80" t="n">
-        <v>38358.34</v>
-      </c>
-      <c r="E80" t="n">
-        <v>-3</v>
+        <v>103.9</v>
       </c>
     </row>
     <row r="81">
@@ -1969,10 +1727,7 @@
         <v>108.88</v>
       </c>
       <c r="D81" t="n">
-        <v>46867</v>
-      </c>
-      <c r="E81" t="n">
-        <v>-4</v>
+        <v>101.7</v>
       </c>
     </row>
     <row r="82">
@@ -1988,10 +1743,7 @@
         <v>108.71</v>
       </c>
       <c r="D82" t="n">
-        <v>50105</v>
-      </c>
-      <c r="E82" t="n">
-        <v>-6</v>
+        <v>97</v>
       </c>
     </row>
     <row r="83">
@@ -2007,10 +1759,7 @@
         <v>110.03</v>
       </c>
       <c r="D83" t="n">
-        <v>55614.5</v>
-      </c>
-      <c r="E83" t="n">
-        <v>-7.8</v>
+        <v>102.2</v>
       </c>
     </row>
     <row r="84">
@@ -2026,10 +1775,7 @@
         <v>106.49</v>
       </c>
       <c r="D84" t="n">
-        <v>63588.6</v>
-      </c>
-      <c r="E84" t="n">
-        <v>-6.2</v>
+        <v>106.3</v>
       </c>
     </row>
     <row r="85">
@@ -2045,10 +1791,7 @@
         <v>103.27</v>
       </c>
       <c r="D85" t="n">
-        <v>73959.89999999999</v>
-      </c>
-      <c r="E85" t="n">
-        <v>-5.4</v>
+        <v>101.3</v>
       </c>
     </row>
     <row r="86">
@@ -2064,10 +1807,7 @@
         <v>117.38</v>
       </c>
       <c r="D86" t="n">
-        <v>17999.7</v>
-      </c>
-      <c r="E86" t="n">
-        <v>4.3</v>
+        <v>102.5</v>
       </c>
     </row>
     <row r="87">
@@ -2083,10 +1823,7 @@
         <v>121.29</v>
       </c>
       <c r="D87" t="n">
-        <v>19924</v>
-      </c>
-      <c r="E87" t="n">
-        <v>4.3</v>
+        <v>100.9</v>
       </c>
     </row>
     <row r="88">
@@ -2102,10 +1839,7 @@
         <v>115.97</v>
       </c>
       <c r="D88" t="n">
-        <v>23100.7</v>
-      </c>
-      <c r="E88" t="n">
-        <v>5.1</v>
+        <v>103.3</v>
       </c>
     </row>
     <row r="89">
@@ -2121,10 +1855,7 @@
         <v>102.35</v>
       </c>
       <c r="D89" t="n">
-        <v>26037.7</v>
-      </c>
-      <c r="E89" t="n">
-        <v>5.8</v>
+        <v>109.5</v>
       </c>
     </row>
     <row r="90">
@@ -2140,10 +1871,7 @@
         <v>101.4</v>
       </c>
       <c r="D90" t="n">
-        <v>27739</v>
-      </c>
-      <c r="E90" t="n">
-        <v>6</v>
+        <v>101.7</v>
       </c>
     </row>
     <row r="91">
@@ -2159,10 +1887,7 @@
         <v>86.97</v>
       </c>
       <c r="D91" t="n">
-        <v>28386</v>
-      </c>
-      <c r="E91" t="n">
-        <v>5.9</v>
+        <v>101.1</v>
       </c>
     </row>
     <row r="92">
@@ -2178,10 +1903,7 @@
         <v>99.2</v>
       </c>
       <c r="D92" t="n">
-        <v>29969</v>
-      </c>
-      <c r="E92" t="n">
-        <v>5.1</v>
+        <v>94</v>
       </c>
     </row>
     <row r="93">
@@ -2197,10 +1919,7 @@
         <v>107.35</v>
       </c>
       <c r="D93" t="n">
-        <v>32237</v>
-      </c>
-      <c r="E93" t="n">
-        <v>3.9</v>
+        <v>97.90000000000001</v>
       </c>
     </row>
     <row r="94">
@@ -2216,10 +1935,7 @@
         <v>109.03</v>
       </c>
       <c r="D94" t="n">
-        <v>32318.25</v>
-      </c>
-      <c r="E94" t="n">
-        <v>3.4</v>
+        <v>97.90000000000001</v>
       </c>
     </row>
     <row r="95">
@@ -2235,10 +1951,7 @@
         <v>116.51</v>
       </c>
       <c r="D95" t="n">
-        <v>39115</v>
-      </c>
-      <c r="E95" t="n">
-        <v>1.6</v>
+        <v>99.3</v>
       </c>
     </row>
     <row r="96">
@@ -2254,10 +1967,7 @@
         <v>118.53</v>
       </c>
       <c r="D96" t="n">
-        <v>41800</v>
-      </c>
-      <c r="E96" t="n">
-        <v>0.9</v>
+        <v>99.09999999999999</v>
       </c>
     </row>
     <row r="97">
@@ -2273,10 +1983,7 @@
         <v>120.6</v>
       </c>
       <c r="D97" t="n">
-        <v>45610.4</v>
-      </c>
-      <c r="E97" t="n">
-        <v>-1.5</v>
+        <v>100.5</v>
       </c>
     </row>
     <row r="98">
@@ -2292,10 +1999,7 @@
         <v>110.1</v>
       </c>
       <c r="D98" t="n">
-        <v>53495.3</v>
-      </c>
-      <c r="E98" t="n">
-        <v>-1</v>
+        <v>106.9</v>
       </c>
     </row>
     <row r="99">
@@ -2311,10 +2015,7 @@
         <v>115.87</v>
       </c>
       <c r="D99" t="n">
-        <v>61564.6</v>
-      </c>
-      <c r="E99" t="n">
-        <v>-1.3</v>
+        <v>102.5</v>
       </c>
     </row>
     <row r="100">
@@ -2330,10 +2031,7 @@
         <v>102.28</v>
       </c>
       <c r="D100" t="n">
-        <v>28708</v>
-      </c>
-      <c r="E100" t="n">
-        <v>7</v>
+        <v>102.9</v>
       </c>
     </row>
     <row r="101">
@@ -2349,10 +2047,7 @@
         <v>104.75</v>
       </c>
       <c r="D101" t="n">
-        <v>34051.5</v>
-      </c>
-      <c r="E101" t="n">
-        <v>7.7</v>
+        <v>103.4</v>
       </c>
     </row>
     <row r="102">
@@ -2368,10 +2063,7 @@
         <v>115.88</v>
       </c>
       <c r="D102" t="n">
-        <v>39915.6</v>
-      </c>
-      <c r="E102" t="n">
-        <v>8.5</v>
+        <v>105.9</v>
       </c>
     </row>
     <row r="103">
@@ -2387,10 +2079,7 @@
         <v>107.66</v>
       </c>
       <c r="D103" t="n">
-        <v>46542</v>
-      </c>
-      <c r="E103" t="n">
-        <v>8.800000000000001</v>
+        <v>103.5</v>
       </c>
     </row>
     <row r="104">
@@ -2406,10 +2095,7 @@
         <v>111.16</v>
       </c>
       <c r="D104" t="n">
-        <v>51111</v>
-      </c>
-      <c r="E104" t="n">
-        <v>9.199999999999999</v>
+        <v>100.8</v>
       </c>
     </row>
     <row r="105">
@@ -2425,10 +2111,7 @@
         <v>99.69</v>
       </c>
       <c r="D105" t="n">
-        <v>54631</v>
-      </c>
-      <c r="E105" t="n">
-        <v>8.5</v>
+        <v>100.4</v>
       </c>
     </row>
     <row r="106">
@@ -2444,10 +2127,7 @@
         <v>96.02</v>
       </c>
       <c r="D106" t="n">
-        <v>59000</v>
-      </c>
-      <c r="E106" t="n">
-        <v>7.5</v>
+        <v>97.7</v>
       </c>
     </row>
     <row r="107">
@@ -2463,10 +2143,7 @@
         <v>94.86</v>
       </c>
       <c r="D107" t="n">
-        <v>62206</v>
-      </c>
-      <c r="E107" t="n">
-        <v>6.4</v>
+        <v>99.5</v>
       </c>
     </row>
     <row r="108">
@@ -2482,10 +2159,7 @@
         <v>102.29</v>
       </c>
       <c r="D108" t="n">
-        <v>60824.68</v>
-      </c>
-      <c r="E108" t="n">
-        <v>5.8</v>
+        <v>103</v>
       </c>
     </row>
     <row r="109">
@@ -2501,10 +2175,7 @@
         <v>116.49</v>
       </c>
       <c r="D109" t="n">
-        <v>73402</v>
-      </c>
-      <c r="E109" t="n">
-        <v>5.4</v>
+        <v>102.3</v>
       </c>
     </row>
     <row r="110">
@@ -2520,10 +2191,7 @@
         <v>103.31</v>
       </c>
       <c r="D110" t="n">
-        <v>77178</v>
-      </c>
-      <c r="E110" t="n">
-        <v>4.1</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="111">
@@ -2539,10 +2207,7 @@
         <v>104.2</v>
       </c>
       <c r="D111" t="n">
-        <v>84471.8</v>
-      </c>
-      <c r="E111" t="n">
-        <v>1.7</v>
+        <v>104</v>
       </c>
     </row>
     <row r="112">
@@ -2558,10 +2223,7 @@
         <v>112.26</v>
       </c>
       <c r="D112" t="n">
-        <v>96728.3</v>
-      </c>
-      <c r="E112" t="n">
-        <v>3.5</v>
+        <v>106.7</v>
       </c>
     </row>
     <row r="113">
@@ -2577,10 +2239,7 @@
         <v>102.99</v>
       </c>
       <c r="D113" t="n">
-        <v>110230.3</v>
-      </c>
-      <c r="E113" t="n">
-        <v>3.4</v>
+        <v>108.5</v>
       </c>
     </row>
     <row r="114">
@@ -2596,10 +2255,7 @@
         <v>100.51</v>
       </c>
       <c r="D114" t="n">
-        <v>35847.9</v>
-      </c>
-      <c r="E114" t="n">
-        <v>-2.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="115">
@@ -2615,10 +2271,7 @@
         <v>101.85</v>
       </c>
       <c r="D115" t="n">
-        <v>38770.7</v>
-      </c>
-      <c r="E115" t="n">
-        <v>-2.4</v>
+        <v>96.90000000000001</v>
       </c>
     </row>
     <row r="116">
@@ -2634,10 +2287,7 @@
         <v>108.06</v>
       </c>
       <c r="D116" t="n">
-        <v>44207.6</v>
-      </c>
-      <c r="E116" t="n">
-        <v>-1.1</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="117">
@@ -2653,10 +2303,7 @@
         <v>103.33</v>
       </c>
       <c r="D117" t="n">
-        <v>49006.9</v>
-      </c>
-      <c r="E117" t="n">
-        <v>-0.2</v>
+        <v>114</v>
       </c>
     </row>
     <row r="118">
@@ -2672,10 +2319,7 @@
         <v>110.35</v>
       </c>
       <c r="D118" t="n">
-        <v>54896</v>
-      </c>
-      <c r="E118" t="n">
-        <v>0.6</v>
+        <v>103.3</v>
       </c>
     </row>
     <row r="119">
@@ -2691,10 +2335,7 @@
         <v>99.20999999999999</v>
       </c>
       <c r="D119" t="n">
-        <v>61311</v>
-      </c>
-      <c r="E119" t="n">
-        <v>0.4</v>
+        <v>101.6</v>
       </c>
     </row>
     <row r="120">
@@ -2710,10 +2351,7 @@
         <v>103.09</v>
       </c>
       <c r="D120" t="n">
-        <v>64959</v>
-      </c>
-      <c r="E120" t="n">
-        <v>1.1</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="121">
@@ -2729,10 +2367,7 @@
         <v>99.31999999999999</v>
       </c>
       <c r="D121" t="n">
-        <v>68496</v>
-      </c>
-      <c r="E121" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
     </row>
     <row r="122">
@@ -2748,10 +2383,7 @@
         <v>110.71</v>
       </c>
       <c r="D122" t="n">
-        <v>75310.39</v>
-      </c>
-      <c r="E122" t="n">
-        <v>-0.5</v>
+        <v>104.7</v>
       </c>
     </row>
     <row r="123">
@@ -2767,10 +2399,7 @@
         <v>104.5</v>
       </c>
       <c r="D123" t="n">
-        <v>87418</v>
-      </c>
-      <c r="E123" t="n">
-        <v>-0.7</v>
+        <v>105.6</v>
       </c>
     </row>
     <row r="124">
@@ -2786,10 +2415,7 @@
         <v>113.32</v>
       </c>
       <c r="D124" t="n">
-        <v>92518</v>
-      </c>
-      <c r="E124" t="n">
-        <v>-2.3</v>
+        <v>98.59999999999999</v>
       </c>
     </row>
     <row r="125">
@@ -2805,10 +2431,7 @@
         <v>109.17</v>
       </c>
       <c r="D125" t="n">
-        <v>94285</v>
-      </c>
-      <c r="E125" t="n">
-        <v>-4.6</v>
+        <v>99.5</v>
       </c>
     </row>
     <row r="126">
@@ -2824,10 +2447,7 @@
         <v>101.73</v>
       </c>
       <c r="D126" t="n">
-        <v>102683.8</v>
-      </c>
-      <c r="E126" t="n">
-        <v>-3.1</v>
+        <v>105.5</v>
       </c>
     </row>
     <row r="127">
@@ -2843,10 +2463,7 @@
         <v>106.01</v>
       </c>
       <c r="D127" t="n">
-        <v>114360.8</v>
-      </c>
-      <c r="E127" t="n">
-        <v>-3.5</v>
+        <v>103.3</v>
       </c>
     </row>
     <row r="128">
@@ -2862,10 +2479,7 @@
         <v>106.25</v>
       </c>
       <c r="D128" t="n">
-        <v>22656.5</v>
-      </c>
-      <c r="E128" t="n">
-        <v>-1.7</v>
+        <v>104.7</v>
       </c>
     </row>
     <row r="129">
@@ -2881,10 +2495,7 @@
         <v>111.12</v>
       </c>
       <c r="D129" t="n">
-        <v>26155.7</v>
-      </c>
-      <c r="E129" t="n">
-        <v>-1.6</v>
+        <v>97.2</v>
       </c>
     </row>
     <row r="130">
@@ -2900,10 +2511,7 @@
         <v>128.37</v>
       </c>
       <c r="D130" t="n">
-        <v>31076.1</v>
-      </c>
-      <c r="E130" t="n">
-        <v>0.1</v>
+        <v>102.7</v>
       </c>
     </row>
     <row r="131">
@@ -2919,10 +2527,7 @@
         <v>96.76000000000001</v>
       </c>
       <c r="D131" t="n">
-        <v>34132.3</v>
-      </c>
-      <c r="E131" t="n">
-        <v>0.6</v>
+        <v>107.5</v>
       </c>
     </row>
     <row r="132">
@@ -2938,10 +2543,7 @@
         <v>97.09999999999999</v>
       </c>
       <c r="D132" t="n">
-        <v>36781</v>
-      </c>
-      <c r="E132" t="n">
-        <v>0.7</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="133">
@@ -2957,10 +2559,7 @@
         <v>92.52</v>
       </c>
       <c r="D133" t="n">
-        <v>38041</v>
-      </c>
-      <c r="E133" t="n">
-        <v>0.9</v>
+        <v>97.40000000000001</v>
       </c>
     </row>
     <row r="134">
@@ -2976,10 +2575,7 @@
         <v>101.46</v>
       </c>
       <c r="D134" t="n">
-        <v>40109</v>
-      </c>
-      <c r="E134" t="n">
-        <v>0.2</v>
+        <v>95.5</v>
       </c>
     </row>
     <row r="135">
@@ -2995,10 +2591,7 @@
         <v>95.89</v>
       </c>
       <c r="D135" t="n">
-        <v>42465</v>
-      </c>
-      <c r="E135" t="n">
-        <v>-0.9</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="136">
@@ -3014,10 +2607,7 @@
         <v>109.39</v>
       </c>
       <c r="D136" t="n">
-        <v>43157.46</v>
-      </c>
-      <c r="E136" t="n">
-        <v>-1.5</v>
+        <v>101.5</v>
       </c>
     </row>
     <row r="137">
@@ -3033,10 +2623,7 @@
         <v>105.33</v>
       </c>
       <c r="D137" t="n">
-        <v>50213</v>
-      </c>
-      <c r="E137" t="n">
-        <v>-2.4</v>
+        <v>100.7</v>
       </c>
     </row>
     <row r="138">
@@ -3052,10 +2639,7 @@
         <v>107.8</v>
       </c>
       <c r="D138" t="n">
-        <v>53113</v>
-      </c>
-      <c r="E138" t="n">
-        <v>-5.1</v>
+        <v>96.2</v>
       </c>
     </row>
     <row r="139">
@@ -3071,10 +2655,7 @@
         <v>116.74</v>
       </c>
       <c r="D139" t="n">
-        <v>58785.8</v>
-      </c>
-      <c r="E139" t="n">
-        <v>-6.7</v>
+        <v>99.59999999999999</v>
       </c>
     </row>
     <row r="140">
@@ -3090,10 +2671,7 @@
         <v>102.11</v>
       </c>
       <c r="D140" t="n">
-        <v>65896.60000000001</v>
-      </c>
-      <c r="E140" t="n">
-        <v>-4.4</v>
+        <v>105.8</v>
       </c>
     </row>
     <row r="141">
@@ -3109,10 +2687,7 @@
         <v>105.76</v>
       </c>
       <c r="D141" t="n">
-        <v>75227.39999999999</v>
-      </c>
-      <c r="E141" t="n">
-        <v>-4.2</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>